<commit_message>
Descartes e relatórios de descarte feitos
</commit_message>
<xml_diff>
--- a/Coleções/Coleção 3 - Shaka de Virgem/avaliacao_colecao3.xlsx
+++ b/Coleções/Coleção 3 - Shaka de Virgem/avaliacao_colecao3.xlsx
@@ -555,20 +555,76 @@
           <t>tentativa 1 - Shaka(Naruto)(atk1).png</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>spritesheet</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Muda o braço no último frame (D não).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -584,19 +640,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -612,19 +655,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -640,19 +670,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -668,19 +685,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -696,20 +700,76 @@
           <t>tentativa 1 - Shaka(Naruto)(Idle).png</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>spritesheet</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Um frame a menos que a referência (C não, Q5 não).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -725,19 +785,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -753,19 +800,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -781,19 +815,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -809,19 +830,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -837,19 +845,71 @@
           <t>tentativa 1 - Shaka(Naruto)(Walk)(1).jpg</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>spritesheet</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -866,19 +926,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -894,19 +941,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -922,19 +956,6 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -950,20 +971,8 @@
           <t>[a gerar]</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>

</xml_diff>